<commit_message>
Leader-first researcher dedup; parse leaders and varied role headings
Leaders were dropped for most TRGs (name in h2, role headings like 'Leader Group').
TRGs with a detected leader: 14 -> ~230. Dedup now anchors persons on TRG leaders
(canonical name from the leader row, prefix-compatible name variants attached).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VuHePFv7oto5SNMHb2pbjZ
</commit_message>
<xml_diff>
--- a/forms/trg/Formulir_TRG_PharmaEpid.xlsx
+++ b/forms/trg/Formulir_TRG_PharmaEpid.xlsx
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B25" s="7">
-        <f>COUNTA(Anggota!B5:B42)</f>
+        <f>COUNTA(Anggota!B5:B43)</f>
         <v/>
       </c>
     </row>
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="B26" s="7">
-        <f>COUNTA(Anggota!F5:F42)</f>
+        <f>COUNTA(Anggota!F5:F43)</f>
         <v/>
       </c>
     </row>
@@ -820,7 +820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -925,35 +925,39 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>apt. Hardiyanti Syarif, M.Farm</t>
+          <t>apt. Muh. Akbar Bahar, Ph.D</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Lecturers</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>Department of Pharmacy, Faculty of Pharmacy, Hasanuddin University</t>
-        </is>
-      </c>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="n"/>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Clinical Pharmacy</t>
+          <t>Pharmacoepidemiology and Applied Pharmacology</t>
         </is>
       </c>
       <c r="F5" s="12" t="n"/>
       <c r="G5" s="12" t="n"/>
       <c r="H5" s="12" t="n"/>
       <c r="I5" s="12" t="n"/>
-      <c r="J5" s="12" t="n"/>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>0000-0002-6582-5615</t>
+        </is>
+      </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>6856363</t>
-        </is>
-      </c>
-      <c r="L5" s="12" t="n"/>
+          <t>6031606</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>57193859399</t>
+        </is>
+      </c>
       <c r="M5" s="11" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -966,12 +970,12 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>apt. A. Anggriani, M.Clin.Pharm</t>
+          <t>apt. Hardiyanti Syarif, M.Farm</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Lecturers</t>
+          <t>Lecturer</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -988,14 +992,10 @@
       <c r="G6" s="12" t="n"/>
       <c r="H6" s="12" t="n"/>
       <c r="I6" s="12" t="n"/>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
-          <t>0000-0001-9831-4494</t>
-        </is>
-      </c>
+      <c r="J6" s="12" t="n"/>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>6750349</t>
+          <t>6856363</t>
         </is>
       </c>
       <c r="L6" s="12" t="n"/>
@@ -1011,12 +1011,12 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>apt. Anshar Saud, M.Farm</t>
+          <t>apt. A. Anggriani, M.Clin.Pharm</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Lecturers</t>
+          <t>Lecturer</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Social Behavioral and Administrative Pharmacy</t>
+          <t>Clinical Pharmacy</t>
         </is>
       </c>
       <c r="F7" s="12" t="n"/>
@@ -1035,12 +1035,12 @@
       <c r="I7" s="12" t="n"/>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>0000-0003-4864-0624</t>
+          <t>0000-0001-9831-4494</t>
         </is>
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>6021685</t>
+          <t>6750349</t>
         </is>
       </c>
       <c r="L7" s="12" t="n"/>
@@ -1056,22 +1056,22 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Prof. Dr. Csupor Dezső</t>
+          <t>apt. Anshar Saud, M.Farm</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>External Collaborators</t>
+          <t>Lecturer</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Institute of Clinical Pharmacy, University of Szeged, Hungary</t>
+          <t>Department of Pharmacy, Faculty of Pharmacy, Hasanuddin University</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Phytotherapy and Clinical pharmacy</t>
+          <t>Social Behavioral and Administrative Pharmacy</t>
         </is>
       </c>
       <c r="F8" s="12" t="n"/>
@@ -1080,15 +1080,15 @@
       <c r="I8" s="12" t="n"/>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>0000-0002-4088-3333</t>
-        </is>
-      </c>
-      <c r="K8" s="12" t="n"/>
-      <c r="L8" s="11" t="inlineStr">
-        <is>
-          <t>55553742985</t>
-        </is>
-      </c>
+          <t>0000-0003-4864-0624</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>6021685</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="n"/>
       <c r="M8" s="11" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -1101,22 +1101,22 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Dr. Arie Arizandi Kurnianto</t>
+          <t>Prof. Dr. Csupor Dezső</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>External Collaborators</t>
+          <t>External collaborator</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Faculty of Pharmacy, University of Pécs, Hungary</t>
+          <t>Institute of Clinical Pharmacy, University of Szeged, Hungary</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>HTA and Pharmacoeconomics</t>
+          <t>Phytotherapy and Clinical pharmacy</t>
         </is>
       </c>
       <c r="F9" s="12" t="n"/>
@@ -1125,13 +1125,13 @@
       <c r="I9" s="12" t="n"/>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>0000-0002-5779-0934</t>
+          <t>0000-0002-4088-3333</t>
         </is>
       </c>
       <c r="K9" s="12" t="n"/>
       <c r="L9" s="11" t="inlineStr">
         <is>
-          <t>57331042200</t>
+          <t>55553742985</t>
         </is>
       </c>
       <c r="M9" s="11" t="inlineStr">
@@ -1146,22 +1146,22 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Prof. apt. Ivan S. Pradipta, Ph.D</t>
+          <t>Dr. Arie Arizandi Kurnianto</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>External Collaborators</t>
+          <t>External collaborator</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Faculty of Pharmacy, Universitas Padjadjaran, Indonesia</t>
+          <t>Faculty of Pharmacy, University of Pécs, Hungary</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Clinical and Community Pharmacy in Infectious Diseases</t>
+          <t>HTA and Pharmacoeconomics</t>
         </is>
       </c>
       <c r="F10" s="12" t="n"/>
@@ -1170,17 +1170,13 @@
       <c r="I10" s="12" t="n"/>
       <c r="J10" s="11" t="inlineStr">
         <is>
-          <t>0000-0002-7151-0783</t>
-        </is>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
-          <t>65244</t>
-        </is>
-      </c>
+          <t>0000-0002-5779-0934</t>
+        </is>
+      </c>
+      <c r="K10" s="12" t="n"/>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>55652137400</t>
+          <t>57331042200</t>
         </is>
       </c>
       <c r="M10" s="11" t="inlineStr">
@@ -1195,22 +1191,22 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Nur Aizati Athirah Daud, Ph.D</t>
+          <t>Prof. apt. Ivan S. Pradipta, Ph.D</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>External Collaborators</t>
+          <t>External collaborator</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>School of Pharmaceutical Sciences, Universiti Sains Malaysia, Malaysia</t>
+          <t>Faculty of Pharmacy, Universitas Padjadjaran, Indonesia</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Clinical pharmacy, Pharmacogenomics, Women Health Pharmacy</t>
+          <t>Clinical and Community Pharmacy in Infectious Diseases</t>
         </is>
       </c>
       <c r="F11" s="12" t="n"/>
@@ -1219,13 +1215,17 @@
       <c r="I11" s="12" t="n"/>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>0000-0003-4336-9468</t>
-        </is>
-      </c>
-      <c r="K11" s="12" t="n"/>
+          <t>0000-0002-7151-0783</t>
+        </is>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>65244</t>
+        </is>
+      </c>
       <c r="L11" s="11" t="inlineStr">
         <is>
-          <t>56226378900</t>
+          <t>55652137400</t>
         </is>
       </c>
       <c r="M11" s="11" t="inlineStr">
@@ -1240,22 +1240,22 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Dr. Felix Chan</t>
+          <t>Nur Aizati Athirah Daud, Ph.D</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>External Collaborators</t>
+          <t>External collaborator</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>School of Health Sciences, University of Birmingham, UK</t>
+          <t>School of Pharmaceutical Sciences, Universiti Sains Malaysia, Malaysia</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Pharmacology, Neuroscience</t>
+          <t>Clinical pharmacy, Pharmacogenomics, Women Health Pharmacy</t>
         </is>
       </c>
       <c r="F12" s="12" t="n"/>
@@ -1264,13 +1264,13 @@
       <c r="I12" s="12" t="n"/>
       <c r="J12" s="11" t="inlineStr">
         <is>
-          <t>0000-0002-4867-9636</t>
+          <t>0000-0003-4336-9468</t>
         </is>
       </c>
       <c r="K12" s="12" t="n"/>
       <c r="L12" s="11" t="inlineStr">
         <is>
-          <t>56956319800</t>
+          <t>56226378900</t>
         </is>
       </c>
       <c r="M12" s="11" t="inlineStr">
@@ -1285,31 +1285,39 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>apt. Dzulfiana Ashan, M.Si</t>
+          <t>Dr. Felix Chan</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Researchers</t>
+          <t>External collaborator</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Department of Pharmacy, Faculty of Pharmacy, Hasanuddin University</t>
+          <t>School of Health Sciences, University of Birmingham, UK</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Clinical Pharmacy</t>
+          <t>Pharmacology, Neuroscience</t>
         </is>
       </c>
       <c r="F13" s="12" t="n"/>
       <c r="G13" s="12" t="n"/>
       <c r="H13" s="12" t="n"/>
       <c r="I13" s="12" t="n"/>
-      <c r="J13" s="12" t="n"/>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>0000-0002-4867-9636</t>
+        </is>
+      </c>
       <c r="K13" s="12" t="n"/>
-      <c r="L13" s="12" t="n"/>
+      <c r="L13" s="11" t="inlineStr">
+        <is>
+          <t>56956319800</t>
+        </is>
+      </c>
       <c r="M13" s="11" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -1322,43 +1330,31 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>apt. Ida Adhayanti, M.Sc</t>
+          <t>apt. Dzulfiana Ashan, M.Si</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Researcher</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Doctoral Program in Pharmacy</t>
+          <t>Department of Pharmacy, Faculty of Pharmacy, Hasanuddin University</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Project: "Drug Use in Pregnancy: Clinical and Pharmacoepidemiological Perspectives”</t>
+          <t>Clinical Pharmacy</t>
         </is>
       </c>
       <c r="F14" s="12" t="n"/>
       <c r="G14" s="12" t="n"/>
       <c r="H14" s="12" t="n"/>
       <c r="I14" s="12" t="n"/>
-      <c r="J14" s="11" t="inlineStr">
-        <is>
-          <t>0000-0003-1997-5820</t>
-        </is>
-      </c>
-      <c r="K14" s="11" t="inlineStr">
-        <is>
-          <t>6181040</t>
-        </is>
-      </c>
-      <c r="L14" s="11" t="inlineStr">
-        <is>
-          <t>58534790900</t>
-        </is>
-      </c>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="12" t="n"/>
+      <c r="L14" s="12" t="n"/>
       <c r="M14" s="11" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -1371,12 +1367,12 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>apt. Madania, M.Sc</t>
+          <t>apt. Ida Adhayanti, M.Sc</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
@@ -1386,7 +1382,7 @@
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Project: "Optimization of Pediatric Tuberculosis Care in Gorontalo: Barriers, Costs, and QoL"</t>
+          <t>Project: "Drug Use in Pregnancy: Clinical and Pharmacoepidemiological Perspectives”</t>
         </is>
       </c>
       <c r="F15" s="12" t="n"/>
@@ -1395,17 +1391,17 @@
       <c r="I15" s="12" t="n"/>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>0000-0002-9296-9286</t>
+          <t>0000-0003-1997-5820</t>
         </is>
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>6657054</t>
+          <t>6181040</t>
         </is>
       </c>
       <c r="L15" s="11" t="inlineStr">
         <is>
-          <t>57220208416</t>
+          <t>58534790900</t>
         </is>
       </c>
       <c r="M15" s="11" t="inlineStr">
@@ -1420,31 +1416,43 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>apt. Annisa Amalanda, S.Farm</t>
+          <t>apt. Madania, M.Sc</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Master’s Program in Pharmacy</t>
+          <t>Doctoral Program in Pharmacy</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Project: "Determinants of Quality of Life in Indonesian Myasthenia Gravis Patients"</t>
+          <t>Project: "Optimization of Pediatric Tuberculosis Care in Gorontalo: Barriers, Costs, and QoL"</t>
         </is>
       </c>
       <c r="F16" s="12" t="n"/>
       <c r="G16" s="12" t="n"/>
       <c r="H16" s="12" t="n"/>
       <c r="I16" s="12" t="n"/>
-      <c r="J16" s="12" t="n"/>
-      <c r="K16" s="12" t="n"/>
-      <c r="L16" s="12" t="n"/>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>0000-0002-9296-9286</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
+        <is>
+          <t>6657054</t>
+        </is>
+      </c>
+      <c r="L16" s="11" t="inlineStr">
+        <is>
+          <t>57220208416</t>
+        </is>
+      </c>
       <c r="M16" s="11" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -1457,12 +1465,12 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>apt. Nurdin, S.Farm</t>
+          <t>apt. Annisa Amalanda, S.Farm</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -1472,7 +1480,7 @@
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Project: "Pharmacists and Herbal Medicines: Attitudes, Barriers, and Information Sources in Community Pharmacies"</t>
+          <t>Project: "Determinants of Quality of Life in Indonesian Myasthenia Gravis Patients"</t>
         </is>
       </c>
       <c r="F17" s="12" t="n"/>
@@ -1494,12 +1502,12 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>apt. Hermin, S.Si</t>
+          <t>apt. Nurdin, S.Farm</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1509,7 +1517,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Project: "CAM Use and Its Impact on Adherence and Quality of Life in Schizophrenia"</t>
+          <t>Project: "Pharmacists and Herbal Medicines: Attitudes, Barriers, and Information Sources in Community Pharmacies"</t>
         </is>
       </c>
       <c r="F18" s="12" t="n"/>
@@ -1531,12 +1539,12 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>apt. Nurhalisa, S.Si</t>
+          <t>apt. Hermin, S.Si</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
@@ -1546,7 +1554,7 @@
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Project: "Medication Adherence and Quality of Life in Thyroid Patients"</t>
+          <t>Project: "CAM Use and Its Impact on Adherence and Quality of Life in Schizophrenia"</t>
         </is>
       </c>
       <c r="F19" s="12" t="n"/>
@@ -1568,12 +1576,12 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>apt. Abd. Rauf Rum, S.Farm</t>
+          <t>apt. Nurhalisa, S.Si</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -1583,7 +1591,7 @@
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Project: "Complementary and Alternative Medicine Use among Hypertension Patients in Community Health Centers"</t>
+          <t>Project: "Medication Adherence and Quality of Life in Thyroid Patients"</t>
         </is>
       </c>
       <c r="F20" s="12" t="n"/>
@@ -1605,12 +1613,12 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>apt. Pratiwi Ningsi, S.Farm</t>
+          <t>apt. Abd. Rauf Rum, S.Farm</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
@@ -1620,7 +1628,7 @@
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>Project: "Indonesian Pharmacists’ Knowledge, Attitudes, and Perceptions of Pharmacogenomics"</t>
+          <t>Project: "Complementary and Alternative Medicine Use among Hypertension Patients in Community Health Centers"</t>
         </is>
       </c>
       <c r="F21" s="12" t="n"/>
@@ -1642,12 +1650,12 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>apt. Adinda Juliawaty, S.Farm</t>
+          <t>apt. Pratiwi Ningsi, S.Farm</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -1657,7 +1665,7 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Project: "CAM Use, Medication Adherence, and Quality of Life in People with HIV/AIDS"</t>
+          <t>Project: "Indonesian Pharmacists’ Knowledge, Attitudes, and Perceptions of Pharmacogenomics"</t>
         </is>
       </c>
       <c r="F22" s="12" t="n"/>
@@ -1679,12 +1687,12 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>apt. Indra Purnama Sari, S.Farm</t>
+          <t>apt. Adinda Juliawaty, S.Farm</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -1694,7 +1702,7 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>Project: "Willingness to Pay for Home Pharmacy Care among Prolanis BPJS Patients"</t>
+          <t>Project: "CAM Use, Medication Adherence, and Quality of Life in People with HIV/AIDS"</t>
         </is>
       </c>
       <c r="F23" s="12" t="n"/>
@@ -1716,12 +1724,12 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>apt. Sitti Nur Alim Kuraisy, S.Si</t>
+          <t>apt. Indra Purnama Sari, S.Farm</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -1731,7 +1739,7 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>Project: "Pattern of Antiepileptic Use and Risk Factors for Drug-Resistant Epilepsy in Adults"</t>
+          <t>Project: "Willingness to Pay for Home Pharmacy Care among Prolanis BPJS Patients"</t>
         </is>
       </c>
       <c r="F24" s="12" t="n"/>
@@ -1753,12 +1761,12 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>apt. Nurul Hikmah Ashri, S.Farm</t>
+          <t>apt. Sitti Nur Alim Kuraisy, S.Si</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
@@ -1768,7 +1776,7 @@
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>Project: "Barriers to Implementing Pharmaceutical Care in Indonesian Community Pharmacies"</t>
+          <t>Project: "Pattern of Antiepileptic Use and Risk Factors for Drug-Resistant Epilepsy in Adults"</t>
         </is>
       </c>
       <c r="F25" s="12" t="n"/>
@@ -1790,22 +1798,22 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>apt. Rahmah Mustarin, MPH</t>
+          <t>apt. Nurul Hikmah Ashri, S.Farm</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Doctoral Program in Pharmacy</t>
+          <t>Master’s Program in Pharmacy</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Project: "Pharmacoeconomic Analysis of Actual Costs and Willingness to Pay for Stunting Care in South Sulawesi"</t>
+          <t>Project: "Barriers to Implementing Pharmaceutical Care in Indonesian Community Pharmacies"</t>
         </is>
       </c>
       <c r="F26" s="12" t="n"/>
@@ -1827,22 +1835,22 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>apt. Abd. Rakhmat Muzakkir, S.Si</t>
+          <t>apt. Rahmah Mustarin, MPH</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Master’s Program in Pharmacy</t>
+          <t>Doctoral Program in Pharmacy</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>Project: "Burden and Resistance of Antibiotic Use Over Five Years in an Indonesian Teaching Hospital"</t>
+          <t>Project: "Pharmacoeconomic Analysis of Actual Costs and Willingness to Pay for Stunting Care in South Sulawesi"</t>
         </is>
       </c>
       <c r="F27" s="12" t="n"/>
@@ -1864,12 +1872,12 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>apt. Destia Risnovianti, S.Si</t>
+          <t>apt. Abd. Rakhmat Muzakkir, S.Si</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -1879,7 +1887,7 @@
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Project: "Evaluation of Community Pharmacists’ Knowledge, Attitudes, Perceptions, and Practices Toward the Management of Common Menstrual Problems in Indonesia""</t>
+          <t>Project: "Burden and Resistance of Antibiotic Use Over Five Years in an Indonesian Teaching Hospital"</t>
         </is>
       </c>
       <c r="F28" s="12" t="n"/>
@@ -1901,12 +1909,12 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>apt. Iftitah Ahmad, S.Farm</t>
+          <t>apt. Destia Risnovianti, S.Si</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
@@ -1916,7 +1924,7 @@
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>Project: "Evaluation of Community Pharmacists’ Competence in the Identification and Management of Malnourished Patients in Indonesia: Perspectives for Improving Nutritional Care Services"</t>
+          <t>Project: "Evaluation of Community Pharmacists’ Knowledge, Attitudes, Perceptions, and Practices Toward the Management of Common Menstrual Problems in Indonesia""</t>
         </is>
       </c>
       <c r="F29" s="12" t="n"/>
@@ -1938,12 +1946,12 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>apt. Muammar Khadafi Burhan, S.Farm</t>
+          <t>apt. Iftitah Ahmad, S.Farm</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -1953,7 +1961,7 @@
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Project: "Association Between Complementary Medicine Use, Medication Adherence, and Quality of Life Among Patients with Epilepsy"</t>
+          <t>Project: "Evaluation of Community Pharmacists’ Competence in the Identification and Management of Malnourished Patients in Indonesia: Perspectives for Improving Nutritional Care Services"</t>
         </is>
       </c>
       <c r="F30" s="12" t="n"/>
@@ -1973,10 +1981,26 @@
       <c r="A31" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="12" t="n"/>
-      <c r="C31" s="12" t="n"/>
-      <c r="D31" s="12" t="n"/>
-      <c r="E31" s="11" t="n"/>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>apt. Muammar Khadafi Burhan, S.Farm</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Student</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Master’s Program in Pharmacy</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Project: "Association Between Complementary Medicine Use, Medication Adherence, and Quality of Life Among Patients with Epilepsy"</t>
+        </is>
+      </c>
       <c r="F31" s="12" t="n"/>
       <c r="G31" s="12" t="n"/>
       <c r="H31" s="12" t="n"/>
@@ -1984,7 +2008,11 @@
       <c r="J31" s="12" t="n"/>
       <c r="K31" s="12" t="n"/>
       <c r="L31" s="12" t="n"/>
-      <c r="M31" s="12" t="n"/>
+      <c r="M31" s="11" t="inlineStr">
+        <is>
+          <t>Aktif</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -2173,15 +2201,32 @@
       <c r="L42" s="12" t="n"/>
       <c r="M42" s="12" t="n"/>
     </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="12" t="n"/>
+      <c r="C43" s="12" t="n"/>
+      <c r="D43" s="12" t="n"/>
+      <c r="E43" s="11" t="n"/>
+      <c r="F43" s="12" t="n"/>
+      <c r="G43" s="12" t="n"/>
+      <c r="H43" s="12" t="n"/>
+      <c r="I43" s="12" t="n"/>
+      <c r="J43" s="12" t="n"/>
+      <c r="K43" s="12" t="n"/>
+      <c r="L43" s="12" t="n"/>
+      <c r="M43" s="12" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:M2"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="F5:H42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Daftar!$A$2:$A$39</formula1>
     </dataValidation>
-    <dataValidation sqref="M5:M42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M5:M43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Daftar!$C$2:$C$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>